<commit_message>
by hussain ...... HIRA TEchnosoft
</commit_message>
<xml_diff>
--- a/web/src/main/webapp/StorageYard/Other/UserDoc/EmployeeRegistration/Employee.xlsx
+++ b/web/src/main/webapp/StorageYard/Other/UserDoc/EmployeeRegistration/Employee.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
     <workbookView xWindow="360" yWindow="120" windowWidth="11340" windowHeight="7500" tabRatio="601"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
   <si>
     <t>Employee Name</t>
   </si>
@@ -52,9 +52,6 @@
     <t>Employee ID</t>
   </si>
   <si>
-    <t>Zydex Location</t>
-  </si>
-  <si>
     <t>Work Location</t>
   </si>
   <si>
@@ -103,12 +100,6 @@
     <t>Experience on Date Of Joining:Month</t>
   </si>
   <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>Vadodara</t>
-  </si>
-  <si>
     <t>Bank Name</t>
   </si>
   <si>
@@ -131,16 +122,43 @@
   </si>
   <si>
     <t>Employee Type</t>
+  </si>
+  <si>
+    <t>Basic Salary</t>
+  </si>
+  <si>
+    <t>ConveysAmount</t>
+  </si>
+  <si>
+    <t>EsicNo</t>
+  </si>
+  <si>
+    <t>TdsAmount</t>
+  </si>
+  <si>
+    <t>Payment</t>
+  </si>
+  <si>
+    <t>PFNo</t>
+  </si>
+  <si>
+    <t>UANO</t>
+  </si>
+  <si>
+    <t>Employee Subtype</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Location</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -153,6 +171,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -187,10 +212,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -219,8 +245,12 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -543,7 +573,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:effectLst>
                 <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="808080"/>
@@ -585,7 +615,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:effectLst>
                 <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="808080"/>
@@ -604,9 +634,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK2"/>
-  <sheetFormatPr defaultRowHeight="21" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AT2"/>
+  <sheetFormatPr defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -645,10 +675,16 @@
     <col min="35" max="35" width="20.140625" style="1" customWidth="1"/>
     <col min="36" max="36" width="14.7109375" style="1" customWidth="1"/>
     <col min="37" max="37" width="19.42578125" style="1" customWidth="1"/>
-    <col min="38" max="16384" width="9.140625" style="1"/>
+    <col min="38" max="38" width="13.5703125" style="1" customWidth="1"/>
+    <col min="39" max="39" width="13.7109375" style="1" customWidth="1"/>
+    <col min="40" max="40" width="14.7109375" style="1" customWidth="1"/>
+    <col min="41" max="41" width="13.140625" style="1" customWidth="1"/>
+    <col min="42" max="44" width="9.140625" style="1"/>
+    <col min="45" max="45" width="12.140625" style="1" customWidth="1"/>
+    <col min="46" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" s="9" customFormat="1" ht="21" customHeight="1">
+    <row r="1" spans="1:46" s="9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>11</v>
       </c>
@@ -659,7 +695,7 @@
         <v>8</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>6</v>
@@ -668,22 +704,22 @@
         <v>7</v>
       </c>
       <c r="G1" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="I1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>16</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>17</v>
       </c>
       <c r="M1" s="8" t="s">
         <v>1</v>
@@ -707,84 +743,133 @@
         <v>9</v>
       </c>
       <c r="T1" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="U1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="V1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="8" t="s">
+      <c r="W1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="8" t="s">
+      <c r="X1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="Y1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="8" t="s">
+      <c r="Z1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="8" t="s">
+      <c r="AA1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" s="8" t="s">
+      <c r="AD1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="AC1" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AE1" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF1" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG1" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="AE1" s="9" t="s">
+      <c r="AH1" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="AF1" s="9" t="s">
+      <c r="AI1" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="AG1" s="9" t="s">
+      <c r="AJ1" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="AH1" s="9" t="s">
+      <c r="AK1" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="AI1" s="9" t="s">
+      <c r="AL1" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="AJ1" s="9" t="s">
+      <c r="AM1" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="AK1" s="9" t="s">
+      <c r="AN1" s="9" t="s">
         <v>38</v>
       </c>
+      <c r="AO1" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP1" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="AQ1" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="AR1" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="AS1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="AT1" s="9" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="2" spans="1:37" s="4" customFormat="1" ht="21" customHeight="1">
-      <c r="A2" s="5"/>
+    <row r="2" spans="1:46" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="6"/>
+      <c r="B2" s="7"/>
       <c r="C2" s="6"/>
-      <c r="D2" s="5"/>
-      <c r="F2" s="5"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="6"/>
       <c r="G2" s="6"/>
-      <c r="H2" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="H2" s="6"/>
       <c r="I2" s="7"/>
-      <c r="K2" s="5"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="6"/>
       <c r="L2" s="7"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
-      <c r="Q2" s="5" t="s">
-        <v>29</v>
-      </c>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="7"/>
       <c r="S2" s="7"/>
-      <c r="AA2" s="5">
-        <v>41</v>
-      </c>
-      <c r="AB2" s="5">
-        <v>5</v>
-      </c>
+      <c r="T2" s="7"/>
+      <c r="U2" s="7"/>
+      <c r="W2" s="7"/>
+      <c r="X2" s="7"/>
+      <c r="Y2" s="7"/>
+      <c r="Z2" s="7"/>
+      <c r="AA2" s="5"/>
+      <c r="AB2" s="5"/>
+      <c r="AC2" s="7"/>
+      <c r="AD2" s="7"/>
+      <c r="AE2" s="7"/>
+      <c r="AF2" s="7"/>
+      <c r="AG2" s="7"/>
+      <c r="AH2" s="7"/>
+      <c r="AI2" s="7"/>
+      <c r="AJ2" s="7"/>
+      <c r="AK2" s="7"/>
+      <c r="AL2" s="7"/>
+      <c r="AM2" s="7"/>
+      <c r="AN2" s="7"/>
+      <c r="AO2" s="7"/>
+      <c r="AP2" s="7"/>
+      <c r="AQ2" s="7"/>
+      <c r="AR2" s="7"/>
+      <c r="AS2" s="7"/>
+      <c r="AT2" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>